<commit_message>
Workbook: dissolve group D, keep the cheap controls, drop MOMENT
A0 stays -- the classical-feature rows are the cheapest insurance in the
table (CPU-minutes) against the critique literature's first attack, and if
handcrafted features beat us on a core corpus we need to be first to know.

Group D dissolves: the random-init row was really the frozen-probe control
(gate 4 of the attribution protocol) and now sits inside the PACLock block
as "冻结探针, 随机初始化", paired with the v2 probe row -- it is the
probe_rand arm already running, zero extra cost. MOMENT is dropped to a
deferred note in the README: a generic TS-FM control defends the B-group
FMs' pretraining value, not our tokenizer claim, and its integration cost
is real -- an easy rebuttal-time addition if asked.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/PACLock_baseline_matrix.xlsx
+++ b/results/PACLock_baseline_matrix.xlsx
@@ -547,21 +547,21 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>D  对照（通用时序 FM；随机初始化同架构 —— 四道归因门第 4 门）</t>
+          <t>缓议：MOMENT 等通用时序 FM 对照 —— 不承重于 tokenizer 主张，留作 rebuttal 期选项</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>E  PACLock（scratch / 预训练 v2 / 冻结探针）</t>
+          <t>D  PACLock（scratch / 预训练 v2 / 冻结探针 vs 随机初始化探针 —— 四道门第 4 门）</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>F  参考值（灰）：无公开权重或异管线论文自报数，只作上下文</t>
+          <t>E  参考值（灰）：无公开权重或异管线论文自报数，只作上下文</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -938,17 +938,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>D 对照</t>
+          <t>D PACLock</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MOMENT (通用时序 FM)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>EEG 特异性对照</t>
+          <t>PACLock (duplex, scratch)</t>
         </is>
       </c>
     </row>
@@ -956,24 +951,25 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PACLock (随机初始化)</t>
+          <t>PACLock (duplex, 预训练 v2)</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>四道门第 4 门</t>
+          <t>band_norm_pac 目标</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>E PACLock</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PACLock (duplex, scratch)</t>
+          <t>PACLock (冻结探针, v2)</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>patch_len 200；表征质量协议</t>
         </is>
       </c>
     </row>
@@ -981,30 +977,17 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PACLock (duplex, 预训练 v2)</t>
+          <t>PACLock (冻结探针, 随机初始化)</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>band_norm_pac 目标</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>PACLock (冻结探针, v2)</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>patch_len 200；表征质量协议</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+          <t>四道门第 4 门对照</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>空单元格 = 尚未跑；单 seed 数字标注 (1 seed)、斜体灰 —— 进论文正表需 3 seed（硬规则 4）</t>
         </is>
@@ -1021,7 +1004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1321,17 +1304,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>D 对照</t>
+          <t>D PACLock</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MOMENT (通用时序 FM)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>EEG 特异性对照</t>
+          <t>PACLock (duplex, scratch)</t>
         </is>
       </c>
     </row>
@@ -1339,24 +1317,25 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PACLock (随机初始化)</t>
+          <t>PACLock (duplex, 预训练 v2)</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>四道门第 4 门</t>
+          <t>band_norm_pac 目标</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>E PACLock</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PACLock (duplex, scratch)</t>
+          <t>PACLock (冻结探针, v2)</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>patch_len 200；表征质量协议</t>
         </is>
       </c>
     </row>
@@ -1364,30 +1343,17 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PACLock (duplex, 预训练 v2)</t>
+          <t>PACLock (冻结探针, 随机初始化)</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>band_norm_pac 目标</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>PACLock (冻结探针, v2)</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>patch_len 200；表征质量协议</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+          <t>四道门第 4 门对照</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>空单元格 = 尚未跑；单 seed 数字标注 (1 seed)、斜体灰 —— 进论文正表需 3 seed（硬规则 4）</t>
         </is>
@@ -1404,7 +1370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1704,17 +1670,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>D 对照</t>
+          <t>D PACLock</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MOMENT (通用时序 FM)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>EEG 特异性对照</t>
+          <t>PACLock (duplex, scratch)</t>
         </is>
       </c>
     </row>
@@ -1722,24 +1683,25 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PACLock (随机初始化)</t>
+          <t>PACLock (duplex, 预训练 v2)</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>四道门第 4 门</t>
+          <t>band_norm_pac 目标</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>E PACLock</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PACLock (duplex, scratch)</t>
+          <t>PACLock (冻结探针, v2)</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>patch_len 200；表征质量协议</t>
         </is>
       </c>
     </row>
@@ -1747,30 +1709,17 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PACLock (duplex, 预训练 v2)</t>
+          <t>PACLock (冻结探针, 随机初始化)</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>band_norm_pac 目标</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>PACLock (冻结探针, v2)</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>patch_len 200；表征质量协议</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+          <t>四道门第 4 门对照</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>空单元格 = 尚未跑；单 seed 数字标注 (1 seed)、斜体灰 —— 进论文正表需 3 seed（硬规则 4）</t>
         </is>
@@ -1787,7 +1736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2087,17 +2036,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>D 对照</t>
+          <t>D PACLock</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MOMENT (通用时序 FM)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>EEG 特异性对照</t>
+          <t>PACLock (duplex, scratch)</t>
         </is>
       </c>
     </row>
@@ -2105,24 +2049,25 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PACLock (随机初始化)</t>
+          <t>PACLock (duplex, 预训练 v2)</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>四道门第 4 门</t>
+          <t>band_norm_pac 目标</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>E PACLock</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PACLock (duplex, scratch)</t>
+          <t>PACLock (冻结探针, v2)</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>patch_len 200；表征质量协议</t>
         </is>
       </c>
     </row>
@@ -2130,30 +2075,17 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PACLock (duplex, 预训练 v2)</t>
+          <t>PACLock (冻结探针, 随机初始化)</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>band_norm_pac 目标</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>PACLock (冻结探针, v2)</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>patch_len 200；表征质量协议</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+          <t>四道门第 4 门对照</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>空单元格 = 尚未跑；单 seed 数字标注 (1 seed)、斜体灰 —— 进论文正表需 3 seed（硬规则 4）</t>
         </is>
@@ -2170,7 +2102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2470,17 +2402,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>D 对照</t>
+          <t>D PACLock</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MOMENT (通用时序 FM)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>EEG 特异性对照</t>
+          <t>PACLock (duplex, scratch)</t>
         </is>
       </c>
     </row>
@@ -2488,24 +2415,25 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PACLock (随机初始化)</t>
+          <t>PACLock (duplex, 预训练 v2)</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>四道门第 4 门</t>
+          <t>band_norm_pac 目标</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>E PACLock</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PACLock (duplex, scratch)</t>
+          <t>PACLock (冻结探针, v2)</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>patch_len 200；表征质量协议</t>
         </is>
       </c>
     </row>
@@ -2513,30 +2441,17 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PACLock (duplex, 预训练 v2)</t>
+          <t>PACLock (冻结探针, 随机初始化)</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>band_norm_pac 目标</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>PACLock (冻结探针, v2)</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>patch_len 200；表征质量协议</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+          <t>四道门第 4 门对照</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>空单元格 = 尚未跑；单 seed 数字标注 (1 seed)、斜体灰 —— 进论文正表需 3 seed（硬规则 4）</t>
         </is>
@@ -2553,7 +2468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2853,17 +2768,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>D 对照</t>
+          <t>D PACLock</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MOMENT (通用时序 FM)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>EEG 特异性对照</t>
+          <t>PACLock (duplex, scratch)</t>
         </is>
       </c>
     </row>
@@ -2871,24 +2781,25 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PACLock (随机初始化)</t>
+          <t>PACLock (duplex, 预训练 v2)</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>四道门第 4 门</t>
+          <t>band_norm_pac 目标</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>E PACLock</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PACLock (duplex, scratch)</t>
+          <t>PACLock (冻结探针, v2)</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>patch_len 200；表征质量协议</t>
         </is>
       </c>
     </row>
@@ -2896,30 +2807,17 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PACLock (duplex, 预训练 v2)</t>
+          <t>PACLock (冻结探针, 随机初始化)</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>band_norm_pac 目标</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>PACLock (冻结探针, v2)</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>patch_len 200；表征质量协议</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+          <t>四道门第 4 门对照</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>空单元格 = 尚未跑；单 seed 数字标注 (1 seed)、斜体灰 —— 进论文正表需 3 seed（硬规则 4）</t>
         </is>
@@ -2936,7 +2834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3236,17 +3134,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>D 对照</t>
+          <t>D PACLock</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MOMENT (通用时序 FM)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>EEG 特异性对照</t>
+          <t>PACLock (duplex, scratch)</t>
         </is>
       </c>
     </row>
@@ -3254,24 +3147,25 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PACLock (随机初始化)</t>
+          <t>PACLock (duplex, 预训练 v2)</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>四道门第 4 门</t>
+          <t>band_norm_pac 目标</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>E PACLock</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PACLock (duplex, scratch)</t>
+          <t>PACLock (冻结探针, v2)</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>patch_len 200；表征质量协议</t>
         </is>
       </c>
     </row>
@@ -3279,30 +3173,17 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PACLock (duplex, 预训练 v2)</t>
+          <t>PACLock (冻结探针, 随机初始化)</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>band_norm_pac 目标</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>PACLock (冻结探针, v2)</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>patch_len 200；表征质量协议</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+          <t>四道门第 4 门对照</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>空单元格 = 尚未跑；单 seed 数字标注 (1 seed)、斜体灰 —— 进论文正表需 3 seed（硬规则 4）</t>
         </is>
@@ -3319,7 +3200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3619,17 +3500,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>D 对照</t>
+          <t>D PACLock</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MOMENT (通用时序 FM)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>EEG 特异性对照</t>
+          <t>PACLock (duplex, scratch)</t>
         </is>
       </c>
     </row>
@@ -3637,24 +3513,25 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PACLock (随机初始化)</t>
+          <t>PACLock (duplex, 预训练 v2)</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>四道门第 4 门</t>
+          <t>band_norm_pac 目标</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>E PACLock</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PACLock (duplex, scratch)</t>
+          <t>PACLock (冻结探针, v2)</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>patch_len 200；表征质量协议</t>
         </is>
       </c>
     </row>
@@ -3662,30 +3539,17 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PACLock (duplex, 预训练 v2)</t>
+          <t>PACLock (冻结探针, 随机初始化)</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>band_norm_pac 目标</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>PACLock (冻结探针, v2)</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>patch_len 200；表征质量协议</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+          <t>四道门第 4 门对照</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>空单元格 = 尚未跑；单 seed 数字标注 (1 seed)、斜体灰 —— 进论文正表需 3 seed（硬规则 4）</t>
         </is>
@@ -3702,7 +3566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4002,17 +3866,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>D 对照</t>
+          <t>D PACLock</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MOMENT (通用时序 FM)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>EEG 特异性对照</t>
+          <t>PACLock (duplex, scratch)</t>
         </is>
       </c>
     </row>
@@ -4020,24 +3879,25 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PACLock (随机初始化)</t>
+          <t>PACLock (duplex, 预训练 v2)</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>四道门第 4 门</t>
+          <t>band_norm_pac 目标</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>E PACLock</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PACLock (duplex, scratch)</t>
+          <t>PACLock (冻结探针, v2)</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>patch_len 200；表征质量协议</t>
         </is>
       </c>
     </row>
@@ -4045,30 +3905,17 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PACLock (duplex, 预训练 v2)</t>
+          <t>PACLock (冻结探针, 随机初始化)</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>band_norm_pac 目标</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>PACLock (冻结探针, v2)</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>patch_len 200；表征质量协议</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+          <t>四道门第 4 门对照</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>空单元格 = 尚未跑；单 seed 数字标注 (1 seed)、斜体灰 —— 进论文正表需 3 seed（硬规则 4）</t>
         </is>
@@ -4085,7 +3932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4378,17 +4225,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>D 对照</t>
+          <t>D PACLock</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MOMENT (通用时序 FM)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>EEG 特异性对照</t>
+          <t>PACLock (duplex, scratch)</t>
         </is>
       </c>
     </row>
@@ -4396,24 +4238,25 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PACLock (随机初始化)</t>
+          <t>PACLock (duplex, 预训练 v2)</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>四道门第 4 门</t>
+          <t>band_norm_pac 目标</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>E PACLock</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PACLock (duplex, scratch)</t>
+          <t>PACLock (冻结探针, v2)</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>patch_len 200；表征质量协议</t>
         </is>
       </c>
     </row>
@@ -4421,71 +4264,58 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PACLock (duplex, 预训练 v2)</t>
+          <t>PACLock (冻结探针, 随机初始化)</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>band_norm_pac 目标</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>PACLock (冻结探针, v2)</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>patch_len 200；表征质量协议</t>
+          <t>四道门第 4 门对照</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>E 参考值（论文自报，不同管线，不可直接比）</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>CodeBrain (ICLR'26, 自报)</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>0.6912</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>F 参考值（论文自报，不同管线，不可直接比）</t>
-        </is>
-      </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>CodeBrain (ICLR'26, 自报)</t>
+          <t>Uni-NTFM-large (ICLR'26, 自报)</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>0.6912</t>
+          <t>0.7030</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Uni-NTFM-large (ICLR'26, 自报)</t>
+          <t>CBraMod (原论文自报)</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>0.7030</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="6" t="inlineStr">
-        <is>
-          <t>CBraMod (原论文自报)</t>
-        </is>
-      </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
           <t>0.6512</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="6" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>空单元格 = 尚未跑；单 seed 数字标注 (1 seed)、斜体灰 —— 进论文正表需 3 seed（硬规则 4）</t>
         </is>
@@ -4502,7 +4332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4795,17 +4625,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>D 对照</t>
+          <t>D PACLock</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MOMENT (通用时序 FM)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>EEG 特异性对照</t>
+          <t>PACLock (duplex, scratch)</t>
         </is>
       </c>
     </row>
@@ -4813,24 +4638,25 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PACLock (随机初始化)</t>
+          <t>PACLock (duplex, 预训练 v2)</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>四道门第 4 门</t>
+          <t>band_norm_pac 目标</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>E PACLock</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PACLock (duplex, scratch)</t>
+          <t>PACLock (冻结探针, v2)</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>patch_len 200；表征质量协议</t>
         </is>
       </c>
     </row>
@@ -4838,30 +4664,17 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PACLock (duplex, 预训练 v2)</t>
+          <t>PACLock (冻结探针, 随机初始化)</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>band_norm_pac 目标</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>PACLock (冻结探针, v2)</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>patch_len 200；表征质量协议</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+          <t>四道门第 4 门对照</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>空单元格 = 尚未跑；单 seed 数字标注 (1 seed)、斜体灰 —— 进论文正表需 3 seed（硬规则 4）</t>
         </is>
@@ -4878,7 +4691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5176,17 +4989,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>D 对照</t>
+          <t>D PACLock</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MOMENT (通用时序 FM)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>EEG 特异性对照</t>
+          <t>PACLock (duplex, scratch)</t>
         </is>
       </c>
     </row>
@@ -5194,24 +5002,25 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PACLock (随机初始化)</t>
+          <t>PACLock (duplex, 预训练 v2)</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>四道门第 4 门</t>
+          <t>band_norm_pac 目标</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>E PACLock</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PACLock (duplex, scratch)</t>
+          <t>PACLock (冻结探针, v2)</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>patch_len 200；表征质量协议</t>
         </is>
       </c>
     </row>
@@ -5219,30 +5028,17 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PACLock (duplex, 预训练 v2)</t>
+          <t>PACLock (冻结探针, 随机初始化)</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>band_norm_pac 目标</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>PACLock (冻结探针, v2)</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>patch_len 200；表征质量协议</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+          <t>四道门第 4 门对照</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>空单元格 = 尚未跑；单 seed 数字标注 (1 seed)、斜体灰 —— 进论文正表需 3 seed（硬规则 4）</t>
         </is>
@@ -5259,7 +5055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5559,17 +5355,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>D 对照</t>
+          <t>D PACLock</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MOMENT (通用时序 FM)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>EEG 特异性对照</t>
+          <t>PACLock (duplex, scratch)</t>
         </is>
       </c>
     </row>
@@ -5577,24 +5368,25 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PACLock (随机初始化)</t>
+          <t>PACLock (duplex, 预训练 v2)</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>四道门第 4 门</t>
+          <t>band_norm_pac 目标</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>E PACLock</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PACLock (duplex, scratch)</t>
+          <t>PACLock (冻结探针, v2)</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>patch_len 200；表征质量协议</t>
         </is>
       </c>
     </row>
@@ -5602,30 +5394,17 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PACLock (duplex, 预训练 v2)</t>
+          <t>PACLock (冻结探针, 随机初始化)</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>band_norm_pac 目标</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>PACLock (冻结探针, v2)</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>patch_len 200；表征质量协议</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+          <t>四道门第 4 门对照</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>空单元格 = 尚未跑；单 seed 数字标注 (1 seed)、斜体灰 —— 进论文正表需 3 seed（硬规则 4）</t>
         </is>
@@ -5642,7 +5421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5935,17 +5714,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>D 对照</t>
+          <t>D PACLock</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MOMENT (通用时序 FM)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>EEG 特异性对照</t>
+          <t>PACLock (duplex, scratch)</t>
         </is>
       </c>
     </row>
@@ -5953,24 +5727,25 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PACLock (随机初始化)</t>
+          <t>PACLock (duplex, 预训练 v2)</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>四道门第 4 门</t>
+          <t>band_norm_pac 目标</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>E PACLock</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PACLock (duplex, scratch)</t>
+          <t>PACLock (冻结探针, v2)</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>patch_len 200；表征质量协议</t>
         </is>
       </c>
     </row>
@@ -5978,30 +5753,17 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PACLock (duplex, 预训练 v2)</t>
+          <t>PACLock (冻结探针, 随机初始化)</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>band_norm_pac 目标</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>PACLock (冻结探针, v2)</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>patch_len 200；表征质量协议</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+          <t>四道门第 4 门对照</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>空单元格 = 尚未跑；单 seed 数字标注 (1 seed)、斜体灰 —— 进论文正表需 3 seed（硬规则 4）</t>
         </is>
@@ -6018,7 +5780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6316,17 +6078,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>D 对照</t>
+          <t>D PACLock</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MOMENT (通用时序 FM)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>EEG 特异性对照</t>
+          <t>PACLock (duplex, scratch)</t>
         </is>
       </c>
     </row>
@@ -6334,24 +6091,25 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PACLock (随机初始化)</t>
+          <t>PACLock (duplex, 预训练 v2)</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>四道门第 4 门</t>
+          <t>band_norm_pac 目标</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>E PACLock</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PACLock (duplex, scratch)</t>
+          <t>PACLock (冻结探针, v2)</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>patch_len 200；表征质量协议</t>
         </is>
       </c>
     </row>
@@ -6359,71 +6117,58 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PACLock (duplex, 预训练 v2)</t>
+          <t>PACLock (冻结探针, 随机初始化)</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>band_norm_pac 目标</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>PACLock (冻结探针, v2)</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>patch_len 200；表征质量协议</t>
+          <t>四道门第 4 门对照</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>E 参考值（论文自报，不同管线，不可直接比）</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>CodeBrain (ICLR'26, 自报)</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>0.8294</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>F 参考值（论文自报，不同管线，不可直接比）</t>
-        </is>
-      </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>CodeBrain (ICLR'26, 自报)</t>
+          <t>Uni-NTFM-large (ICLR'26, 自报)</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>0.8294</t>
+          <t>0.8197</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Uni-NTFM-large (ICLR'26, 自报)</t>
+          <t>REVE-Base (原论文自报)</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>0.8197</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="6" t="inlineStr">
-        <is>
-          <t>REVE-Base (原论文自报)</t>
-        </is>
-      </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
           <t>0.8315</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="6" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>空单元格 = 尚未跑；单 seed 数字标注 (1 seed)、斜体灰 —— 进论文正表需 3 seed（硬规则 4）</t>
         </is>
@@ -6440,7 +6185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6733,17 +6478,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>D 对照</t>
+          <t>D PACLock</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MOMENT (通用时序 FM)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>EEG 特异性对照</t>
+          <t>PACLock (duplex, scratch)</t>
         </is>
       </c>
     </row>
@@ -6751,24 +6491,25 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PACLock (随机初始化)</t>
+          <t>PACLock (duplex, 预训练 v2)</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>四道门第 4 门</t>
+          <t>band_norm_pac 目标</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>E PACLock</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PACLock (duplex, scratch)</t>
+          <t>PACLock (冻结探针, v2)</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>patch_len 200；表征质量协议</t>
         </is>
       </c>
     </row>
@@ -6776,30 +6517,17 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PACLock (duplex, 预训练 v2)</t>
+          <t>PACLock (冻结探针, 随机初始化)</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>band_norm_pac 目标</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>PACLock (冻结探针, v2)</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>patch_len 200；表征质量协议</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+          <t>四道门第 4 门对照</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>空单元格 = 尚未跑；单 seed 数字标注 (1 seed)、斜体灰 —— 进论文正表需 3 seed（硬规则 4）</t>
         </is>
@@ -6816,7 +6544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -7116,17 +6844,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>D 对照</t>
+          <t>D PACLock</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MOMENT (通用时序 FM)</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>EEG 特异性对照</t>
+          <t>PACLock (duplex, scratch)</t>
         </is>
       </c>
     </row>
@@ -7134,24 +6857,25 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PACLock (随机初始化)</t>
+          <t>PACLock (duplex, 预训练 v2)</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>四道门第 4 门</t>
+          <t>band_norm_pac 目标</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>E PACLock</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PACLock (duplex, scratch)</t>
+          <t>PACLock (冻结探针, v2)</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>patch_len 200；表征质量协议</t>
         </is>
       </c>
     </row>
@@ -7159,42 +6883,29 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PACLock (duplex, 预训练 v2)</t>
+          <t>PACLock (冻结探针, 随机初始化)</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>band_norm_pac 目标</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>PACLock (冻结探针, v2)</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>patch_len 200；表征质量协议</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>F 参考值（论文自报，不同管线，不可直接比）</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
+          <t>四道门第 4 门对照</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>E 参考值（论文自报，不同管线，不可直接比）</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>CEEDNet (数据集作者, NeuroImage'23)</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>空单元格 = 尚未跑；单 seed 数字标注 (1 seed)、斜体灰 —— 进论文正表需 3 seed（硬规则 4）</t>
         </is>

</xml_diff>